<commit_message>
Agrega semana 14-19/9: data periodo, manejo digestivo (amoxicilina+B12), regenera PDF/excels/panel
</commit_message>
<xml_diff>
--- a/excel/01_glucosa.xlsx
+++ b/excel/01_glucosa.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,17 +413,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D360"/>
+  <dimension ref="A1:D372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
@@ -7625,6 +7621,246 @@
       <c r="D360" t="inlineStr">
         <is>
           <t>orig29</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>300</v>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>193</v>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>276</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>193</v>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>216</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>252</v>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>320</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>143</v>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>301</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>172</v>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>medianoche</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>342</v>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>mediodia</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>304</v>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>usuario</t>
         </is>
       </c>
     </row>

</xml_diff>